<commit_message>
fix: décodage des entités HTML dans les titres
</commit_message>
<xml_diff>
--- a/samples/books-demo/clean.xlsx
+++ b/samples/books-demo/clean.xlsx
@@ -819,7 +819,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Shakespeare&amp;#39;s Sonnets</t>
+          <t>Shakespeare's Sonnets</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -871,7 +871,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Scott Pilgrim&amp;#39;s Precious Little Life (Scott Pilgrim #1)</t>
+          <t>Scott Pilgrim's Precious Little Life (Scott Pilgrim #1)</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -1027,7 +1027,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>It&amp;#39;s Only the Himalayas</t>
+          <t>It's Only the Himalayas</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -1209,7 +1209,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>America&amp;#39;s Cradle of Quarterbacks: Western Pennsylvania&amp;#39;s Football Factory from Johnny Unitas to Joe Montana</t>
+          <t>America's Cradle of Quarterbacks: Western Pennsylvania's Football Factory from Johnny Unitas to Joe Montana</t>
         </is>
       </c>
       <c r="B28" s="3" t="n">
@@ -1417,7 +1417,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Sophie&amp;#39;s World</t>
+          <t>Sophie's World</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -1547,7 +1547,7 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>You can&amp;#39;t bury them all: Poems</t>
+          <t>You can't bury them all: Poems</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
@@ -1781,7 +1781,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Unseen City: The Majesty of Pigeons, the Discreet Charm of Snails &amp;amp; Other Wonders of the Urban Wilderness</t>
+          <t>Unseen City: The Majesty of Pigeons, the Discreet Charm of Snails &amp; Other Wonders of the Urban Wilderness</t>
         </is>
       </c>
       <c r="B50" s="3" t="n">
@@ -2145,7 +2145,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>The Most Perfect Thing: Inside (and Outside) a Bird&amp;#39;s Egg</t>
+          <t>The Most Perfect Thing: Inside (and Outside) a Bird's Egg</t>
         </is>
       </c>
       <c r="B64" s="3" t="n">
@@ -2405,7 +2405,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>The Activist&amp;#39;s Tao Te Ching: Ancient Advice for a Modern Revolution</t>
+          <t>The Activist's Tao Te Ching: Ancient Advice for a Modern Revolution</t>
         </is>
       </c>
       <c r="B74" s="3" t="n">

</xml_diff>

<commit_message>
fix: colonne des titres élargie, export PDF sans rognage
</commit_message>
<xml_diff>
--- a/samples/books-demo/clean.xlsx
+++ b/samples/books-demo/clean.xlsx
@@ -485,12 +485,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
@@ -3235,6 +3235,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E101" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId101"/>
   </tableParts>

</xml_diff>